<commit_message>
Add pagination following, anti-bot compliance detection, and human-handoff tier
- Pagination: orchestrator follows next-page links (re-polls the frontier so page
  2→3→… are walked within one run), with a max_pages safety cap and config toggle.
- Compliance: detect anti-bot / access-denied responses (403/401/429 + Cloudflare
  challenge markers); dead-letter with "refusing to evade" instead of extracting from
  or authoring against a challenge page. Verified live: frontierdental.com → 403.
- Human-in-the-loop final escalation tier: when automation can't/shouldn't proceed
  (blocked, or no profile + no LLM, or auto-author failed), queue an actionable
  human-help request (manual_help table) rather than failing silently or evading.
  Surfaced in `safco stats`, the run summary, and relayed by the conductor.
- 3 new tests (pagination walk + max_pages cap, block→handoff). 18 total, all green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716416+00:00</t>
+          <t>2026-06-27T04:08:41.667747+00:00</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716528+00:00</t>
+          <t>2026-06-27T04:08:41.667855+00:00</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716490+00:00</t>
+          <t>2026-06-27T04:08:41.667816+00:00</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716663+00:00</t>
+          <t>2026-06-27T04:08:41.667986+00:00</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.714810+00:00</t>
+          <t>2026-06-27T04:08:41.667657+00:00</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716379+00:00</t>
+          <t>2026-06-27T04:08:41.667720+00:00</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716509+00:00</t>
+          <t>2026-06-27T04:08:41.667836+00:00</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716440+00:00</t>
+          <t>2026-06-27T04:08:41.667771+00:00</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716644+00:00</t>
+          <t>2026-06-27T04:08:41.667968+00:00</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716621+00:00</t>
+          <t>2026-06-27T04:08:41.667950+00:00</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716603+00:00</t>
+          <t>2026-06-27T04:08:41.667932+00:00</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716565+00:00</t>
+          <t>2026-06-27T04:08:41.667892+00:00</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716547+00:00</t>
+          <t>2026-06-27T04:08:41.667873+00:00</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716464+00:00</t>
+          <t>2026-06-27T04:08:41.667793+00:00</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:33.716583+00:00</t>
+          <t>2026-06-27T04:08:41.667911+00:00</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095537+00:00</t>
+          <t>2026-06-27T04:08:42.369880+00:00</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095795+00:00</t>
+          <t>2026-06-27T04:08:42.370122+00:00</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095740+00:00</t>
+          <t>2026-06-27T04:08:42.370071+00:00</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095684+00:00</t>
+          <t>2026-06-27T04:08:42.370017+00:00</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095563+00:00</t>
+          <t>2026-06-27T04:08:42.369903+00:00</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095493+00:00</t>
+          <t>2026-06-27T04:08:42.369840+00:00</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095722+00:00</t>
+          <t>2026-06-27T04:08:42.370053+00:00</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095776+00:00</t>
+          <t>2026-06-27T04:08:42.370105+00:00</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095585+00:00</t>
+          <t>2026-06-27T04:08:42.369925+00:00</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095625+00:00</t>
+          <t>2026-06-27T04:08:42.369963+00:00</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095664+00:00</t>
+          <t>2026-06-27T04:08:42.370000+00:00</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095645+00:00</t>
+          <t>2026-06-27T04:08:42.369982+00:00</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095605+00:00</t>
+          <t>2026-06-27T04:08:42.369944+00:00</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095758+00:00</t>
+          <t>2026-06-27T04:08:42.370088+00:00</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-06-27T02:58:35.095704+00:00</t>
+          <t>2026-06-27T04:08:42.370035+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>